<commit_message>
feat: add horizontal competitor comparison matrices
</commit_message>
<xml_diff>
--- a/assets/matic-detailed-dd-workbench.xlsx
+++ b/assets/matic-detailed-dd-workbench.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页" sheetId="1" r:id="R7dd3530bfed34556"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="调研对象候选库" sheetId="2" r:id="Ra6bc5fc7fc154295"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="联系与访谈进度" sheetId="3" r:id="Rc95632520f254913"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料及专家报告索引" sheetId="4" r:id="R997a6f74eea24e1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="具体产品与方案矩阵" sheetId="5" r:id="Rd6a1874488164dc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="技术路线矩阵" sheetId="6" r:id="R44310487460f4264"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题跟踪表" sheetId="7" r:id="R081139c045c34299"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="结论登记表" sheetId="8" r:id="Rcfc27b0e820a4e75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="专家分歧表" sheetId="9" r:id="R9889d66efadd4051"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一部分入选结论" sheetId="10" r:id="Rf2e06a2e1cb346ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="11" r:id="R9d394371e5704470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页" sheetId="1" r:id="R0facd34715a84d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="调研对象候选库" sheetId="2" r:id="Ra2f699956ab741b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="联系与访谈进度" sheetId="3" r:id="Rd2c72f9876764441"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料及专家报告索引" sheetId="4" r:id="Rceacb0e0b46547d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="具体产品与方案矩阵" sheetId="5" r:id="R8a56d90718c149b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="技术路线矩阵" sheetId="6" r:id="Rd76db2f9feeb4835"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题跟踪表" sheetId="7" r:id="R548a767081d7487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="结论登记表" sheetId="8" r:id="R9bdc77568cbb4eea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="专家分歧表" sheetId="9" r:id="Rfbd86f6c3947471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一部分入选结论" sheetId="10" r:id="R16a2c0e0c4134ae9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="11" r:id="R19fbbc6d20a84b7b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3284,7 +3284,7 @@
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="40" t="str">
-        <x:v>3. 产品/方案与技术路线分别维护；每次更新均检查新对象、新路线、突破价值、路线拥挤度、相对优劣势及比较条件变化。</x:v>
+        <x:v>3. 产品/方案与技术路线分别按证据长表维护；“具体判断”优先写成可直接进入报告单元格的展示值，并记录单位、口径及条件。</x:v>
       </x:c>
       <x:c r="B22" s="40"/>
       <x:c r="C22" s="40"/>
@@ -3296,7 +3296,7 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="40" t="str">
-        <x:v>4. 阶段性或最终报告只在明确指令后生成；成文前检查专家证据门槛、去重和结论历史。</x:v>
+        <x:v>4. 阶段性或最终报告只在明确指令后生成；成文时将有效长表转置为“维度为行、本项目为首列”的横向矩阵。</x:v>
       </x:c>
       <x:c r="B23" s="40"/>
       <x:c r="C23" s="40"/>
@@ -6271,7 +6271,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R686a69f5a9b947d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63c3b873afc04140"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8789,7 +8789,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c5adc88520a4436"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65635cf1bc924474"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12964,7 +12964,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8de48f8cf0624158"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a6233138aa94571"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16746,7 +16746,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reff0fb9e1ccf4b1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18db71ee3f274ff2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20297,7 +20297,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R460e485d3eb64062"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc39f1a7c45124cd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20372,7 +20372,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>每个“产品或方案×对比维度”单独一行并沿用稳定CMP-P编号；直接竞品按临床决策、患者、场景或采购预算重叠判断，注册/上市状态与商业化状态分开记录。</x:v>
+        <x:v>证据长表：每个“产品或方案×对比维度”单独一行并沿用稳定CMP-P编号；“具体判断”填写可进入报告横向矩阵的展示值，数值另注明单位、口径和条件，成文时再按维度转置。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -26750,7 +26750,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeea1a488b8b43c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66412f01b9264838"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26823,7 +26823,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>每个“技术路线×对比维度”单独一行并沿用稳定CMP-R编号；本项目路线必须登记，持续验证突破价值、关键国产替代、路线成熟度、拥挤度和替代关系。</x:v>
+        <x:v>证据长表：每个“技术路线×对比维度”单独一行并沿用稳定CMP-R编号；“具体判断”填写可进入报告横向矩阵的展示值，本项目路线必须登记，成文时再按维度转置。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -32988,7 +32988,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0324d4b562c40fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd48f4097cd734caf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37575,7 +37575,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16ec4e88eab54856"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cba3ff690074732"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41753,7 +41753,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64b7bdf8fe8f448d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5964921815ec4e17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44680,7 +44680,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9793de9ee124441c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb72793439f2a4e4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>